<commit_message>
vault backup: 2026-03-24 16:49:14
</commit_message>
<xml_diff>
--- a/开发平台/codex/项目/人员简历筛选和重组/output/spreadsheet/国开行-企业级风险管理平台-人员简历-整理计划-V1_关联表.xlsx
+++ b/开发平台/codex/项目/人员简历筛选和重组/output/spreadsheet/国开行-企业级风险管理平台-人员简历-整理计划-V1_关联表.xlsx
@@ -8,9 +8,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人员简历整理计划" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人员项目客户关联表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终人员匹配表" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'人员项目客户关联表'!$A$3:$L$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'最终人员匹配表'!$A$3:$L$34</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -2773,4 +2775,2018 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>国开行-企业级风险管理平台-最终人员匹配表</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>说明：该表根据人员清单.xlsx展开到单人粒度，用于最终与整理计划表匹配。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>系统/子系统</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>标准角色</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>人员姓名</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>客户简称</t>
+        </is>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>客户全称</t>
+        </is>
+      </c>
+      <c r="G3" s="28" t="inlineStr">
+        <is>
+          <t>项目名称</t>
+        </is>
+      </c>
+      <c r="H3" s="28" t="inlineStr">
+        <is>
+          <t>项目内容</t>
+        </is>
+      </c>
+      <c r="I3" s="28" t="inlineStr">
+        <is>
+          <t>岗位信息</t>
+        </is>
+      </c>
+      <c r="J3" s="28" t="inlineStr">
+        <is>
+          <t>岗位内容</t>
+        </is>
+      </c>
+      <c r="K3" s="28" t="inlineStr">
+        <is>
+          <t>经验要求摘要</t>
+        </is>
+      </c>
+      <c r="L3" s="28" t="inlineStr">
+        <is>
+          <t>来源</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>业务连续性管理</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t>项目管理岗</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>项目管理岗</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
+          <t>陈亮5</t>
+        </is>
+      </c>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F4" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G4" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H4" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展项目群管理、进度控制、风险识别、资源协调和交付推进。</t>
+        </is>
+      </c>
+      <c r="I4" s="29" t="inlineStr">
+        <is>
+          <t>项目管理岗</t>
+        </is>
+      </c>
+      <c r="J4" s="29" t="inlineStr">
+        <is>
+          <t>负责项目群统筹、计划制定、风险跟踪、跨团队协调和进度推进。</t>
+        </is>
+      </c>
+      <c r="K4" s="29" t="inlineStr">
+        <is>
+          <t>总年限：8年
+银行业系统开发领域项目管理年限：3年</t>
+        </is>
+      </c>
+      <c r="L4" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>业务连续性管理</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>需求分析岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="C5" s="32" t="inlineStr">
+        <is>
+          <t>需求分析岗</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>徐道章</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F5" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G5" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H5" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展需求分析、需求建模、业务流程设计和需求管理。</t>
+        </is>
+      </c>
+      <c r="I5" s="31" t="inlineStr">
+        <is>
+          <t>需求分析岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="J5" s="31" t="inlineStr">
+        <is>
+          <t>负责需求调研、需求建模、流程设计和需求分析。</t>
+        </is>
+      </c>
+      <c r="K5" s="31" t="inlineStr">
+        <is>
+          <t>总年限：7年
+银行业风险管理领域需求分析年限：3年</t>
+        </is>
+      </c>
+      <c r="L5" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>业务连续性管理</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>开发A岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>开发A岗</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>叶中满</t>
+        </is>
+      </c>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F6" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G6" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H6" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展Java/Vue/SpringBoot/SpringCloud开发、信创适配和详细设计。</t>
+        </is>
+      </c>
+      <c r="I6" s="29" t="inlineStr">
+        <is>
+          <t>开发A岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>负责核心模块开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K6" s="29" t="inlineStr">
+        <is>
+          <t>总年限：7年
+银行业系统开发领域开发年限：5年</t>
+        </is>
+      </c>
+      <c r="L6" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>业务连续性管理</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>开发B岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="inlineStr">
+        <is>
+          <t>开发B岗</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>王富</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F7" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H7" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展Java/Vue/SpringBoot/SpringCloud开发、信创适配和详细设计。</t>
+        </is>
+      </c>
+      <c r="I7" s="31" t="inlineStr">
+        <is>
+          <t>开发B岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="J7" s="31" t="inlineStr">
+        <is>
+          <t>负责核心模块开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K7" s="31" t="inlineStr">
+        <is>
+          <t>总年限：7年
+银行业系统开发领域开发年限：5年</t>
+        </is>
+      </c>
+      <c r="L7" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>业务连续性管理</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>测试岗</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>测试岗</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>方伟明</t>
+        </is>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F8" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H8" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展测试用例编写、集成测试、系统测试和缺陷跟踪。</t>
+        </is>
+      </c>
+      <c r="I8" s="29" t="inlineStr">
+        <is>
+          <t>测试岗</t>
+        </is>
+      </c>
+      <c r="J8" s="29" t="inlineStr">
+        <is>
+          <t>负责测试用例设计、集成测试、系统测试和缺陷跟踪。</t>
+        </is>
+      </c>
+      <c r="K8" s="29" t="inlineStr">
+        <is>
+          <t>总年限：8年</t>
+        </is>
+      </c>
+      <c r="L8" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="32" t="inlineStr">
+        <is>
+          <t>业务连续性管理</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>质量控制岗</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>质量控制岗</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>刘蕊3</t>
+        </is>
+      </c>
+      <c r="E9" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F9" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H9" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展质量体系建设、过程改进和质量管控。</t>
+        </is>
+      </c>
+      <c r="I9" s="31" t="inlineStr">
+        <is>
+          <t>质量控制岗</t>
+        </is>
+      </c>
+      <c r="J9" s="31" t="inlineStr">
+        <is>
+          <t>负责质量体系建设、过程改进和质量问题跟踪。</t>
+        </is>
+      </c>
+      <c r="K9" s="31" t="inlineStr">
+        <is>
+          <t>总年限：8年</t>
+        </is>
+      </c>
+      <c r="L9" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>业务连续性管理</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>王欣11</t>
+        </is>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G10" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H10" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规开发交付。</t>
+        </is>
+      </c>
+      <c r="I10" s="29" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="J10" s="29" t="inlineStr">
+        <is>
+          <t>负责Java开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K10" s="29" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="32" t="inlineStr">
+        <is>
+          <t>业务连续性管理</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="D11" s="32" t="inlineStr">
+        <is>
+          <t>张浩强</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H11" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规开发交付。</t>
+        </is>
+      </c>
+      <c r="I11" s="31" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="J11" s="31" t="inlineStr">
+        <is>
+          <t>负责Java开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K11" s="31" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L11" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>业务连续性管理</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>常规测试岗</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>常规测试岗</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>付鹏</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G12" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H12" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规测试交付。</t>
+        </is>
+      </c>
+      <c r="I12" s="29" t="inlineStr">
+        <is>
+          <t>常规测试岗</t>
+        </is>
+      </c>
+      <c r="J12" s="29" t="inlineStr">
+        <is>
+          <t>负责测试用例设计、集成测试、系统测试和缺陷跟踪。</t>
+        </is>
+      </c>
+      <c r="K12" s="29" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L12" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="32" t="inlineStr">
+        <is>
+          <t>业务连续性管理</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>常规需求岗</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="inlineStr">
+        <is>
+          <t>常规需求岗</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>龚开永</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G13" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H13" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规需求分析。</t>
+        </is>
+      </c>
+      <c r="I13" s="31" t="inlineStr">
+        <is>
+          <t>常规需求岗</t>
+        </is>
+      </c>
+      <c r="J13" s="31" t="inlineStr">
+        <is>
+          <t>负责需求调研、业务建模和需求文档输出。</t>
+        </is>
+      </c>
+      <c r="K13" s="31" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L13" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>风险偏好与内部风险报告</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>项目管理岗</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>项目管理岗</t>
+        </is>
+      </c>
+      <c r="D14" s="30" t="inlineStr">
+        <is>
+          <t>马骏3</t>
+        </is>
+      </c>
+      <c r="E14" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G14" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H14" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展项目群管理、进度控制、风险识别、资源协调和交付推进。</t>
+        </is>
+      </c>
+      <c r="I14" s="29" t="inlineStr">
+        <is>
+          <t>项目管理岗</t>
+        </is>
+      </c>
+      <c r="J14" s="29" t="inlineStr">
+        <is>
+          <t>负责项目群统筹、计划制定、风险跟踪、跨团队协调和进度推进。</t>
+        </is>
+      </c>
+      <c r="K14" s="29" t="inlineStr">
+        <is>
+          <t>总年限：8年
+银行业系统开发领域项目管理年限：3年</t>
+        </is>
+      </c>
+      <c r="L14" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="32" t="inlineStr">
+        <is>
+          <t>风险偏好与内部风险报告</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>需求分析岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="inlineStr">
+        <is>
+          <t>需求分析岗</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>王佩</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G15" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H15" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展需求分析、需求建模、业务流程设计和需求管理。</t>
+        </is>
+      </c>
+      <c r="I15" s="31" t="inlineStr">
+        <is>
+          <t>需求分析岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="J15" s="31" t="inlineStr">
+        <is>
+          <t>负责需求调研、需求建模、流程设计和需求分析。</t>
+        </is>
+      </c>
+      <c r="K15" s="31" t="inlineStr">
+        <is>
+          <t>总年限：7年
+银行业风险管理领域需求分析年限：3年</t>
+        </is>
+      </c>
+      <c r="L15" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>风险偏好与内部风险报告</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>开发A岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>开发A岗</t>
+        </is>
+      </c>
+      <c r="D16" s="30" t="inlineStr">
+        <is>
+          <t>刘承灵</t>
+        </is>
+      </c>
+      <c r="E16" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F16" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G16" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H16" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展Java/Vue/SpringBoot/SpringCloud开发、信创适配和详细设计。</t>
+        </is>
+      </c>
+      <c r="I16" s="29" t="inlineStr">
+        <is>
+          <t>开发A岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="J16" s="29" t="inlineStr">
+        <is>
+          <t>负责核心模块开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K16" s="29" t="inlineStr">
+        <is>
+          <t>总年限：7年
+银行业系统开发领域开发年限：5年</t>
+        </is>
+      </c>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="32" t="inlineStr">
+        <is>
+          <t>风险偏好与内部风险报告</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="inlineStr">
+        <is>
+          <t>开发B岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="C17" s="32" t="inlineStr">
+        <is>
+          <t>开发B岗</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>邓力群</t>
+        </is>
+      </c>
+      <c r="E17" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G17" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H17" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展Java/Vue/SpringBoot/SpringCloud开发、信创适配和详细设计。</t>
+        </is>
+      </c>
+      <c r="I17" s="31" t="inlineStr">
+        <is>
+          <t>开发B岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="J17" s="31" t="inlineStr">
+        <is>
+          <t>负责核心模块开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K17" s="31" t="inlineStr">
+        <is>
+          <t>总年限：7年
+银行业系统开发领域开发年限：5年</t>
+        </is>
+      </c>
+      <c r="L17" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>风险偏好与内部风险报告</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>测试岗</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>测试岗</t>
+        </is>
+      </c>
+      <c r="D18" s="30" t="inlineStr">
+        <is>
+          <t>贺湘黔</t>
+        </is>
+      </c>
+      <c r="E18" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G18" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H18" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展测试用例编写、集成测试、系统测试和缺陷跟踪。</t>
+        </is>
+      </c>
+      <c r="I18" s="29" t="inlineStr">
+        <is>
+          <t>测试岗</t>
+        </is>
+      </c>
+      <c r="J18" s="29" t="inlineStr">
+        <is>
+          <t>负责测试用例设计、集成测试、系统测试和缺陷跟踪。</t>
+        </is>
+      </c>
+      <c r="K18" s="29" t="inlineStr">
+        <is>
+          <t>总年限：8年</t>
+        </is>
+      </c>
+      <c r="L18" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>风险偏好与内部风险报告</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>质量控制岗</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>质量控制岗</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>彭赤瑰</t>
+        </is>
+      </c>
+      <c r="E19" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G19" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H19" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展质量体系建设、过程改进和质量管控。</t>
+        </is>
+      </c>
+      <c r="I19" s="31" t="inlineStr">
+        <is>
+          <t>质量控制岗</t>
+        </is>
+      </c>
+      <c r="J19" s="31" t="inlineStr">
+        <is>
+          <t>负责质量体系建设、过程改进和质量问题跟踪。</t>
+        </is>
+      </c>
+      <c r="K19" s="31" t="inlineStr">
+        <is>
+          <t>总年限：8年</t>
+        </is>
+      </c>
+      <c r="L19" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>风险偏好与内部风险报告</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="inlineStr">
+        <is>
+          <t>叶顺斌</t>
+        </is>
+      </c>
+      <c r="E20" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F20" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G20" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H20" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规开发交付。</t>
+        </is>
+      </c>
+      <c r="I20" s="29" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="J20" s="29" t="inlineStr">
+        <is>
+          <t>负责Java开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K20" s="29" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L20" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="32" t="inlineStr">
+        <is>
+          <t>风险偏好与内部风险报告</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="D21" s="32" t="inlineStr">
+        <is>
+          <t>刘璇3</t>
+        </is>
+      </c>
+      <c r="E21" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F21" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G21" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H21" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规开发交付。</t>
+        </is>
+      </c>
+      <c r="I21" s="31" t="inlineStr">
+        <is>
+          <t>常规开发岗</t>
+        </is>
+      </c>
+      <c r="J21" s="31" t="inlineStr">
+        <is>
+          <t>负责Java开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K21" s="31" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L21" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>风险偏好与内部风险报告</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>常规测试岗</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>常规测试岗</t>
+        </is>
+      </c>
+      <c r="D22" s="30" t="inlineStr">
+        <is>
+          <t>曲桂才</t>
+        </is>
+      </c>
+      <c r="E22" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F22" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G22" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H22" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规测试交付。</t>
+        </is>
+      </c>
+      <c r="I22" s="29" t="inlineStr">
+        <is>
+          <t>常规测试岗</t>
+        </is>
+      </c>
+      <c r="J22" s="29" t="inlineStr">
+        <is>
+          <t>负责测试用例设计、集成测试、系统测试和缺陷跟踪。</t>
+        </is>
+      </c>
+      <c r="K22" s="29" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L22" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
+          <t>风险偏好与内部风险报告</t>
+        </is>
+      </c>
+      <c r="B23" s="31" t="inlineStr">
+        <is>
+          <t>常规需求岗</t>
+        </is>
+      </c>
+      <c r="C23" s="32" t="inlineStr">
+        <is>
+          <t>常规需求岗</t>
+        </is>
+      </c>
+      <c r="D23" s="32" t="inlineStr">
+        <is>
+          <t>田王浩</t>
+        </is>
+      </c>
+      <c r="E23" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F23" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G23" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H23" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规需求分析。</t>
+        </is>
+      </c>
+      <c r="I23" s="31" t="inlineStr">
+        <is>
+          <t>常规需求岗</t>
+        </is>
+      </c>
+      <c r="J23" s="31" t="inlineStr">
+        <is>
+          <t>负责需求调研、业务建模和需求文档输出。</t>
+        </is>
+      </c>
+      <c r="K23" s="31" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L23" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>压力测试</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>项目管理岗</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>项目管理岗</t>
+        </is>
+      </c>
+      <c r="D24" s="30" t="inlineStr">
+        <is>
+          <t>秦鹏帅</t>
+        </is>
+      </c>
+      <c r="E24" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F24" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G24" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展项目群管理、进度控制、风险识别、资源协调和交付推进。</t>
+        </is>
+      </c>
+      <c r="I24" s="29" t="inlineStr">
+        <is>
+          <t>项目管理岗</t>
+        </is>
+      </c>
+      <c r="J24" s="29" t="inlineStr">
+        <is>
+          <t>负责项目群统筹、计划制定、风险跟踪、跨团队协调和进度推进。</t>
+        </is>
+      </c>
+      <c r="K24" s="29" t="inlineStr">
+        <is>
+          <t>总年限：8年
+银行业系统开发领域项目管理年限：3年</t>
+        </is>
+      </c>
+      <c r="L24" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="32" t="inlineStr">
+        <is>
+          <t>压力测试</t>
+        </is>
+      </c>
+      <c r="B25" s="31" t="inlineStr">
+        <is>
+          <t>需求分析岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="inlineStr">
+        <is>
+          <t>需求分析岗</t>
+        </is>
+      </c>
+      <c r="D25" s="32" t="inlineStr">
+        <is>
+          <t>李文帅</t>
+        </is>
+      </c>
+      <c r="E25" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F25" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G25" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H25" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展需求分析、需求建模、业务流程设计和需求管理。</t>
+        </is>
+      </c>
+      <c r="I25" s="31" t="inlineStr">
+        <is>
+          <t>需求分析岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="J25" s="31" t="inlineStr">
+        <is>
+          <t>负责需求调研、需求建模、流程设计和需求分析。</t>
+        </is>
+      </c>
+      <c r="K25" s="31" t="inlineStr">
+        <is>
+          <t>总年限：7年
+银行业风险管理领域需求分析年限：3年</t>
+        </is>
+      </c>
+      <c r="L25" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>压力测试</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>开发A岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="C26" s="30" t="inlineStr">
+        <is>
+          <t>开发A岗</t>
+        </is>
+      </c>
+      <c r="D26" s="30" t="inlineStr">
+        <is>
+          <t>宋兴盛1</t>
+        </is>
+      </c>
+      <c r="E26" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F26" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G26" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H26" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展Java/Vue/SpringBoot/SpringCloud开发、信创适配和详细设计。</t>
+        </is>
+      </c>
+      <c r="I26" s="29" t="inlineStr">
+        <is>
+          <t>开发A岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="J26" s="29" t="inlineStr">
+        <is>
+          <t>负责核心模块开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K26" s="29" t="inlineStr">
+        <is>
+          <t>总年限：7年
+银行业系统开发领域开发年限：5年</t>
+        </is>
+      </c>
+      <c r="L26" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="32" t="inlineStr">
+        <is>
+          <t>压力测试</t>
+        </is>
+      </c>
+      <c r="B27" s="31" t="inlineStr">
+        <is>
+          <t>开发B岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="inlineStr">
+        <is>
+          <t>开发B岗</t>
+        </is>
+      </c>
+      <c r="D27" s="32" t="inlineStr">
+        <is>
+          <t>李楠楠</t>
+        </is>
+      </c>
+      <c r="E27" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F27" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G27" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H27" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展Java/Vue/SpringBoot/SpringCloud开发、信创适配和详细设计。</t>
+        </is>
+      </c>
+      <c r="I27" s="31" t="inlineStr">
+        <is>
+          <t>开发B岗（风险管理领域）</t>
+        </is>
+      </c>
+      <c r="J27" s="31" t="inlineStr">
+        <is>
+          <t>负责核心模块开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K27" s="31" t="inlineStr">
+        <is>
+          <t>总年限：7年
+银行业系统开发领域开发年限：5年</t>
+        </is>
+      </c>
+      <c r="L27" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>压力测试</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="inlineStr">
+        <is>
+          <t>测试岗</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr">
+        <is>
+          <t>测试岗</t>
+        </is>
+      </c>
+      <c r="D28" s="30" t="inlineStr">
+        <is>
+          <t>郭玉春</t>
+        </is>
+      </c>
+      <c r="E28" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F28" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G28" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H28" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展测试用例编写、集成测试、系统测试和缺陷跟踪。</t>
+        </is>
+      </c>
+      <c r="I28" s="29" t="inlineStr">
+        <is>
+          <t>测试岗</t>
+        </is>
+      </c>
+      <c r="J28" s="29" t="inlineStr">
+        <is>
+          <t>负责测试用例设计、集成测试、系统测试和缺陷跟踪。</t>
+        </is>
+      </c>
+      <c r="K28" s="29" t="inlineStr">
+        <is>
+          <t>总年限：8年</t>
+        </is>
+      </c>
+      <c r="L28" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="32" t="inlineStr">
+        <is>
+          <t>压力测试</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="inlineStr">
+        <is>
+          <t>质量控制岗</t>
+        </is>
+      </c>
+      <c r="C29" s="32" t="inlineStr">
+        <is>
+          <t>质量控制岗</t>
+        </is>
+      </c>
+      <c r="D29" s="32" t="inlineStr">
+        <is>
+          <t>柯晓敏</t>
+        </is>
+      </c>
+      <c r="E29" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F29" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G29" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H29" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展质量体系建设、过程改进和质量管控。</t>
+        </is>
+      </c>
+      <c r="I29" s="31" t="inlineStr">
+        <is>
+          <t>质量控制岗</t>
+        </is>
+      </c>
+      <c r="J29" s="31" t="inlineStr">
+        <is>
+          <t>负责质量体系建设、过程改进和质量问题跟踪。</t>
+        </is>
+      </c>
+      <c r="K29" s="31" t="inlineStr">
+        <is>
+          <t>总年限：8年</t>
+        </is>
+      </c>
+      <c r="L29" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>压力测试</t>
+        </is>
+      </c>
+      <c r="B30" s="29" t="inlineStr">
+        <is>
+          <t>常规-需求</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="inlineStr">
+        <is>
+          <t>常规需求</t>
+        </is>
+      </c>
+      <c r="D30" s="30" t="inlineStr">
+        <is>
+          <t>陶振纲</t>
+        </is>
+      </c>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F30" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G30" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H30" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规需求分析。</t>
+        </is>
+      </c>
+      <c r="I30" s="29" t="inlineStr">
+        <is>
+          <t>常规需求</t>
+        </is>
+      </c>
+      <c r="J30" s="29" t="inlineStr">
+        <is>
+          <t>负责需求调研、业务建模和需求文档输出。</t>
+        </is>
+      </c>
+      <c r="K30" s="29" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L30" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>压力测试</t>
+        </is>
+      </c>
+      <c r="B31" s="31" t="inlineStr">
+        <is>
+          <t>常规-开发</t>
+        </is>
+      </c>
+      <c r="C31" s="32" t="inlineStr">
+        <is>
+          <t>常规开发</t>
+        </is>
+      </c>
+      <c r="D31" s="32" t="inlineStr">
+        <is>
+          <t>高旭2</t>
+        </is>
+      </c>
+      <c r="E31" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F31" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G31" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H31" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规开发交付。</t>
+        </is>
+      </c>
+      <c r="I31" s="31" t="inlineStr">
+        <is>
+          <t>常规开发</t>
+        </is>
+      </c>
+      <c r="J31" s="31" t="inlineStr">
+        <is>
+          <t>负责Java开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K31" s="31" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L31" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>压力测试</t>
+        </is>
+      </c>
+      <c r="B32" s="29" t="inlineStr">
+        <is>
+          <t>常规-开发</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="inlineStr">
+        <is>
+          <t>常规开发</t>
+        </is>
+      </c>
+      <c r="D32" s="30" t="inlineStr">
+        <is>
+          <t>冯佳豪</t>
+        </is>
+      </c>
+      <c r="E32" s="30" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F32" s="30" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G32" s="29" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H32" s="29" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规开发交付。</t>
+        </is>
+      </c>
+      <c r="I32" s="29" t="inlineStr">
+        <is>
+          <t>常规开发</t>
+        </is>
+      </c>
+      <c r="J32" s="29" t="inlineStr">
+        <is>
+          <t>负责Java开发、详细设计、联调测试和上线支持。</t>
+        </is>
+      </c>
+      <c r="K32" s="29" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L32" s="29" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="36" customHeight="1">
+      <c r="A33" s="32" t="inlineStr">
+        <is>
+          <t>压力测试</t>
+        </is>
+      </c>
+      <c r="B33" s="31" t="inlineStr">
+        <is>
+          <t>常规-测试</t>
+        </is>
+      </c>
+      <c r="C33" s="32" t="inlineStr">
+        <is>
+          <t>常规测试</t>
+        </is>
+      </c>
+      <c r="D33" s="32" t="inlineStr">
+        <is>
+          <t>李鹏11</t>
+        </is>
+      </c>
+      <c r="E33" s="32" t="inlineStr">
+        <is>
+          <t>国开行</t>
+        </is>
+      </c>
+      <c r="F33" s="32" t="inlineStr">
+        <is>
+          <t>国家开发银行</t>
+        </is>
+      </c>
+      <c r="G33" s="31" t="inlineStr">
+        <is>
+          <t>企业级风险管理平台</t>
+        </is>
+      </c>
+      <c r="H33" s="31" t="inlineStr">
+        <is>
+          <t>围绕企业级风险管理平台开展常规测试交付。</t>
+        </is>
+      </c>
+      <c r="I33" s="31" t="inlineStr">
+        <is>
+          <t>常规测试</t>
+        </is>
+      </c>
+      <c r="J33" s="31" t="inlineStr">
+        <is>
+          <t>负责测试用例设计、集成测试、系统测试和缺陷跟踪。</t>
+        </is>
+      </c>
+      <c r="K33" s="31" t="inlineStr">
+        <is>
+          <t>总年限：5年
+风险管理领域年限：无要求</t>
+        </is>
+      </c>
+      <c r="L33" s="31" t="inlineStr">
+        <is>
+          <t>人员清单.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="33" t="inlineStr">
+        <is>
+          <t>合计人员数</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="n"/>
+      <c r="C34" s="31" t="n"/>
+      <c r="D34" s="33">
+        <f>COUNTA(D4:D33)</f>
+        <v/>
+      </c>
+      <c r="E34" s="31" t="n"/>
+      <c r="F34" s="31" t="n"/>
+      <c r="G34" s="31" t="n"/>
+      <c r="H34" s="31" t="n"/>
+      <c r="I34" s="31" t="n"/>
+      <c r="J34" s="31" t="n"/>
+      <c r="K34" s="31" t="n"/>
+      <c r="L34" s="31" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:L34"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>